<commit_message>
fix : fix midtrans and change to indonesian language
</commit_message>
<xml_diff>
--- a/data-siswa-50-2.xlsx
+++ b/data-siswa-50-2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROYEK PENELITIAN SPP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Pembayaran_spp\pembayaran_spp\pembayaran_spp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8C1E11F1-3B06-4FA3-8CD2-BEBD9BCCCE2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{868FD0B3-DE85-4613-A57D-0E0B640DA614}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{764C0629-A8AF-41BF-9117-334BE5AB9392}"/>
   </bookViews>
@@ -31,8 +31,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -83,9 +81,6 @@
     <t>ok</t>
   </si>
   <si>
-    <t>Farmasi Klinis Dan Komunitas</t>
-  </si>
-  <si>
     <t>ADE FITRIANI</t>
   </si>
   <si>
@@ -95,9 +90,6 @@
     <t>Adinda Dwi Larasaty</t>
   </si>
   <si>
-    <t>Teknologi Laboratorium Medik</t>
-  </si>
-  <si>
     <t>AFIANA JESSIKA</t>
   </si>
   <si>
@@ -110,9 +102,6 @@
     <t>Ajeng Nindya Pratiwi</t>
   </si>
   <si>
-    <t>Asisten Keperawatan</t>
-  </si>
-  <si>
     <t>AL HAFIZ JUNH</t>
   </si>
   <si>
@@ -240,6 +229,15 @@
   </si>
   <si>
     <t>Perempuan</t>
+  </si>
+  <si>
+    <t>Farmasi</t>
+  </si>
+  <si>
+    <t>Keperawatan</t>
+  </si>
+  <si>
+    <t>Teknik Laboratorium</t>
   </si>
 </sst>
 </file>
@@ -283,14 +281,7 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -305,7 +296,14 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -342,15 +340,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DEF5842F-A883-4D15-A90F-7B9A6FA42762}" name="Table_Table_Sheet1" displayName="Table_Table_Sheet1" ref="A1:I50" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:I50" xr:uid="{DEF5842F-A883-4D15-A90F-7B9A6FA42762}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{A2D9B9E0-533A-479E-9B99-4E6393DEBD7A}" uniqueName="1" name="nama" queryTableFieldId="1" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{A2D9B9E0-533A-479E-9B99-4E6393DEBD7A}" uniqueName="1" name="nama" queryTableFieldId="1" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{929EA0C4-BFAE-4247-A32C-6832A3FC999C}" uniqueName="2" name="nisn" queryTableFieldId="2"/>
-    <tableColumn id="3" xr3:uid="{AD868D46-2D18-4434-B5F5-278AD17DAEE0}" uniqueName="3" name="jenis_kelamin" queryTableFieldId="3" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{AD868D46-2D18-4434-B5F5-278AD17DAEE0}" uniqueName="3" name="jenis_kelamin" queryTableFieldId="3" dataDxfId="3"/>
     <tableColumn id="4" xr3:uid="{671671BC-60D9-4F37-88E3-C3F1F0C70D2A}" uniqueName="4" name="wali_id" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{B9448828-CAE0-4739-8F4F-F1C0574BE8A1}" uniqueName="5" name="wali_status" queryTableFieldId="5" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{480FFB32-6AFC-4170-BC01-7C568D5AC880}" uniqueName="6" name="jurusan" queryTableFieldId="6" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{B9448828-CAE0-4739-8F4F-F1C0574BE8A1}" uniqueName="5" name="wali_status" queryTableFieldId="5" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{480FFB32-6AFC-4170-BC01-7C568D5AC880}" uniqueName="6" name="jurusan" queryTableFieldId="6" dataDxfId="1"/>
     <tableColumn id="7" xr3:uid="{464FDE8F-41C8-4899-B0B4-DB1A52F217CD}" uniqueName="7" name="kelas" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{8F6D1168-0F6F-4C24-B89A-E16EFA772E54}" uniqueName="8" name="angkatan" queryTableFieldId="8"/>
-    <tableColumn id="9" xr3:uid="{D708CF7A-1589-43D4-B92B-EA22AABFD8C8}" uniqueName="9" name="biaya_id" queryTableFieldId="9" dataDxfId="1">
+    <tableColumn id="9" xr3:uid="{D708CF7A-1589-43D4-B92B-EA22AABFD8C8}" uniqueName="9" name="biaya_id" queryTableFieldId="9" dataDxfId="0">
       <calculatedColumnFormula>Table_Table_Sheet1[[#This Row],[angkatan]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -359,9 +357,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -399,7 +397,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -505,7 +503,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -647,7 +645,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -694,7 +692,7 @@
         <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -714,7 +712,7 @@
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G2">
         <v>10</v>
@@ -728,13 +726,13 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>30491220436</v>
       </c>
       <c r="C3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -743,7 +741,7 @@
         <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G3">
         <v>12</v>
@@ -757,13 +755,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4">
         <v>30491321481</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D4">
         <v>4</v>
@@ -772,7 +770,7 @@
         <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G4">
         <v>11</v>
@@ -786,13 +784,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>3034520069</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D5">
         <v>5</v>
@@ -801,7 +799,7 @@
         <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G5">
         <v>12</v>
@@ -815,13 +813,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B6">
         <v>30491221553</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D6">
         <v>6</v>
@@ -830,7 +828,7 @@
         <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G6">
         <v>10</v>
@@ -844,13 +842,13 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B7">
         <v>30491321486</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D7">
         <v>7</v>
@@ -859,7 +857,7 @@
         <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G7">
         <v>11</v>
@@ -873,13 +871,13 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>30491221590</v>
       </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D8">
         <v>8</v>
@@ -888,7 +886,7 @@
         <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G8">
         <v>10</v>
@@ -902,13 +900,13 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B9">
         <v>30141020333</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D9">
         <v>9</v>
@@ -917,7 +915,7 @@
         <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="G9">
         <v>12</v>
@@ -931,7 +929,7 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>30141021384</v>
@@ -946,7 +944,7 @@
         <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="G10">
         <v>10</v>
@@ -960,13 +958,13 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B11">
         <v>30141021404</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D11">
         <v>11</v>
@@ -975,7 +973,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="G11">
         <v>10</v>
@@ -989,7 +987,7 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>3034521103</v>
@@ -1004,7 +1002,7 @@
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G12">
         <v>10</v>
@@ -1018,13 +1016,13 @@
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>3034621078</v>
       </c>
       <c r="C13" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D13">
         <v>13</v>
@@ -1033,7 +1031,7 @@
         <v>10</v>
       </c>
       <c r="F13" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G13">
         <v>11</v>
@@ -1047,13 +1045,13 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B14">
         <v>30491321482</v>
       </c>
       <c r="C14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D14">
         <v>14</v>
@@ -1062,7 +1060,7 @@
         <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G14">
         <v>11</v>
@@ -1076,13 +1074,13 @@
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B15">
         <v>30491220459</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D15">
         <v>15</v>
@@ -1091,7 +1089,7 @@
         <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G15">
         <v>12</v>
@@ -1105,13 +1103,13 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>30491220460</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D16">
         <v>16</v>
@@ -1120,7 +1118,7 @@
         <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G16">
         <v>12</v>
@@ -1134,13 +1132,13 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>30491321483</v>
       </c>
       <c r="C17" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D17">
         <v>17</v>
@@ -1149,7 +1147,7 @@
         <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G17">
         <v>11</v>
@@ -1163,13 +1161,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B18">
         <v>30141021385</v>
       </c>
       <c r="C18" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D18">
         <v>18</v>
@@ -1178,7 +1176,7 @@
         <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="G18">
         <v>10</v>
@@ -1192,13 +1190,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B19">
         <v>30491321484</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D19">
         <v>19</v>
@@ -1207,7 +1205,7 @@
         <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G19">
         <v>11</v>
@@ -1221,13 +1219,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B20">
         <v>30491221554</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D20">
         <v>20</v>
@@ -1236,7 +1234,7 @@
         <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G20">
         <v>10</v>
@@ -1250,13 +1248,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B21">
         <v>30491221591</v>
       </c>
       <c r="C21" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D21">
         <v>21</v>
@@ -1265,7 +1263,7 @@
         <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>11</v>
+        <v>61</v>
       </c>
       <c r="G21">
         <v>10</v>
@@ -1279,7 +1277,7 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B22">
         <v>3034621079</v>
@@ -1294,7 +1292,7 @@
         <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G22">
         <v>11</v>
@@ -1308,13 +1306,13 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B23">
         <v>3034521104</v>
       </c>
       <c r="C23" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D23">
         <v>23</v>
@@ -1323,7 +1321,7 @@
         <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G23">
         <v>10</v>
@@ -1337,13 +1335,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B24">
         <v>3034621080</v>
       </c>
       <c r="C24" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D24">
         <v>24</v>
@@ -1352,7 +1350,7 @@
         <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G24">
         <v>11</v>
@@ -1366,13 +1364,13 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B25">
         <v>30141021405</v>
       </c>
       <c r="C25" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D25">
         <v>25</v>
@@ -1381,7 +1379,7 @@
         <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="G25">
         <v>10</v>
@@ -1395,13 +1393,13 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B26">
         <v>3034520070</v>
       </c>
       <c r="C26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D26">
         <v>26</v>
@@ -1410,7 +1408,7 @@
         <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>15</v>
+        <v>61</v>
       </c>
       <c r="G26">
         <v>12</v>
@@ -1424,13 +1422,13 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B27">
         <v>30141021386</v>
       </c>
       <c r="C27" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D27">
         <v>27</v>
@@ -1439,7 +1437,7 @@
         <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="G27">
         <v>10</v>
@@ -1453,13 +1451,13 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B28">
         <v>30141121364</v>
       </c>
       <c r="C28" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D28">
         <v>28</v>
@@ -1468,7 +1466,7 @@
         <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="G28">
         <v>11</v>
@@ -1482,13 +1480,13 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B29">
         <v>30491220437</v>
       </c>
       <c r="C29" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D29">
         <v>29</v>
@@ -1497,7 +1495,7 @@
         <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="G29">
         <v>12</v>
@@ -1511,13 +1509,13 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B30">
         <v>30141121365</v>
       </c>
       <c r="C30" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D30">
         <v>30</v>
@@ -1526,7 +1524,7 @@
         <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="G30">
         <v>11</v>
@@ -1540,13 +1538,13 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B31">
         <v>30491221555</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D31">
         <v>31</v>
@@ -1555,7 +1553,7 @@
         <v>10</v>
       </c>
       <c r="F31" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="G31">
         <v>10</v>
@@ -1569,13 +1567,13 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B32">
         <v>30491221592</v>
       </c>
       <c r="C32" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D32">
         <v>32</v>
@@ -1584,7 +1582,7 @@
         <v>10</v>
       </c>
       <c r="F32" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="G32">
         <v>10</v>
@@ -1598,13 +1596,13 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B33">
         <v>30491220461</v>
       </c>
       <c r="C33" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D33">
         <v>33</v>
@@ -1613,7 +1611,7 @@
         <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="G33">
         <v>12</v>
@@ -1627,13 +1625,13 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B34">
         <v>30141021406</v>
       </c>
       <c r="C34" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D34">
         <v>34</v>
@@ -1642,7 +1640,7 @@
         <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="G34">
         <v>10</v>
@@ -1656,7 +1654,7 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B35">
         <v>30491221556</v>
@@ -1671,7 +1669,7 @@
         <v>10</v>
       </c>
       <c r="F35" t="s">
-        <v>11</v>
+        <v>62</v>
       </c>
       <c r="G35">
         <v>10</v>
@@ -1685,7 +1683,7 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B36">
         <v>3034621081</v>
@@ -1700,7 +1698,7 @@
         <v>10</v>
       </c>
       <c r="F36" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="G36">
         <v>11</v>
@@ -1714,13 +1712,13 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B37">
         <v>30141021387</v>
       </c>
       <c r="C37" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D37">
         <v>37</v>
@@ -1729,7 +1727,7 @@
         <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="G37">
         <v>10</v>
@@ -1743,7 +1741,7 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B38">
         <v>30141020334</v>
@@ -1758,7 +1756,7 @@
         <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="G38">
         <v>12</v>
@@ -1772,13 +1770,13 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B39">
         <v>3034520071</v>
       </c>
       <c r="C39" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D39">
         <v>39</v>
@@ -1787,7 +1785,7 @@
         <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="G39">
         <v>12</v>
@@ -1801,13 +1799,13 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B40">
         <v>30491220438</v>
       </c>
       <c r="C40" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D40">
         <v>40</v>
@@ -1816,7 +1814,7 @@
         <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G40">
         <v>12</v>
@@ -1830,13 +1828,13 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B41">
         <v>30491321487</v>
       </c>
       <c r="C41" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D41">
         <v>41</v>
@@ -1845,7 +1843,7 @@
         <v>10</v>
       </c>
       <c r="F41" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G41">
         <v>11</v>
@@ -1859,13 +1857,13 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B42">
         <v>3034521105</v>
       </c>
       <c r="C42" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D42">
         <v>42</v>
@@ -1874,7 +1872,7 @@
         <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="G42">
         <v>10</v>
@@ -1888,13 +1886,13 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B43">
         <v>30491220462</v>
       </c>
       <c r="C43" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D43">
         <v>43</v>
@@ -1903,7 +1901,7 @@
         <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G43">
         <v>12</v>
@@ -1917,13 +1915,13 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B44">
         <v>3034621082</v>
       </c>
       <c r="C44" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D44">
         <v>44</v>
@@ -1932,7 +1930,7 @@
         <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>15</v>
+        <v>63</v>
       </c>
       <c r="G44">
         <v>11</v>
@@ -1946,13 +1944,13 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B45">
         <v>30141020335</v>
       </c>
       <c r="C45" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D45">
         <v>45</v>
@@ -1961,7 +1959,7 @@
         <v>10</v>
       </c>
       <c r="F45" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="G45">
         <v>12</v>
@@ -1975,13 +1973,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B46">
         <v>30491321488</v>
       </c>
       <c r="C46" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D46">
         <v>46</v>
@@ -1990,7 +1988,7 @@
         <v>10</v>
       </c>
       <c r="F46" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G46">
         <v>11</v>
@@ -2004,13 +2002,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B47">
         <v>30141020363</v>
       </c>
       <c r="C47" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D47">
         <v>47</v>
@@ -2019,7 +2017,7 @@
         <v>10</v>
       </c>
       <c r="F47" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="G47">
         <v>12</v>
@@ -2033,13 +2031,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B48">
         <v>30491221593</v>
       </c>
       <c r="C48" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D48">
         <v>48</v>
@@ -2048,7 +2046,7 @@
         <v>10</v>
       </c>
       <c r="F48" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G48">
         <v>10</v>
@@ -2062,13 +2060,13 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B49">
         <v>30491221557</v>
       </c>
       <c r="C49" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D49">
         <v>49</v>
@@ -2077,7 +2075,7 @@
         <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G49">
         <v>10</v>
@@ -2091,13 +2089,13 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B50">
         <v>30491221594</v>
       </c>
       <c r="C50" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D50">
         <v>50</v>
@@ -2106,7 +2104,7 @@
         <v>10</v>
       </c>
       <c r="F50" t="s">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="G50">
         <v>10</v>
@@ -2120,7 +2118,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1:H50">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>